<commit_message>
fix: correct Henley Park high zone discount rates to 8.5% and rebuild
</commit_message>
<xml_diff>
--- a/files/九龙-启德-Henley Park.xlsx
+++ b/files/九龙-启德-Henley Park.xlsx
@@ -666,11 +666,11 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="27" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
@@ -22318,18 +22318,18 @@
       </c>
       <c r="J334" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K334" s="5" t="n">
-        <v>13435200</v>
+        <v>13509000</v>
       </c>
       <c r="L334" s="5" t="n">
-        <v>32296</v>
+        <v>32474</v>
       </c>
       <c r="M334" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N334" s="3" t="inlineStr">
@@ -23086,18 +23086,18 @@
       </c>
       <c r="J346" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K346" s="5" t="n">
-        <v>13283200</v>
+        <v>13356200</v>
       </c>
       <c r="L346" s="5" t="n">
-        <v>31931</v>
+        <v>32106</v>
       </c>
       <c r="M346" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N346" s="3" t="inlineStr">
@@ -23846,18 +23846,18 @@
       </c>
       <c r="J358" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K358" s="5" t="n">
-        <v>13207700</v>
+        <v>13280300</v>
       </c>
       <c r="L358" s="5" t="n">
-        <v>31749</v>
+        <v>31924</v>
       </c>
       <c r="M358" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N358" s="3" t="inlineStr">
@@ -24606,18 +24606,18 @@
       </c>
       <c r="J370" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K370" s="5" t="n">
-        <v>13132200</v>
+        <v>13204300</v>
       </c>
       <c r="L370" s="5" t="n">
-        <v>31568</v>
+        <v>31741</v>
       </c>
       <c r="M370" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N370" s="3" t="inlineStr">
@@ -25358,18 +25358,18 @@
       </c>
       <c r="J382" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K382" s="5" t="n">
-        <v>13056600</v>
+        <v>13128400</v>
       </c>
       <c r="L382" s="5" t="n">
-        <v>31386</v>
+        <v>31559</v>
       </c>
       <c r="M382" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N382" s="3" t="inlineStr">
@@ -26110,18 +26110,18 @@
       </c>
       <c r="J394" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K394" s="5" t="n">
-        <v>12981100</v>
+        <v>13052400</v>
       </c>
       <c r="L394" s="5" t="n">
-        <v>31205</v>
+        <v>31376</v>
       </c>
       <c r="M394" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N394" s="3" t="inlineStr">
@@ -26862,18 +26862,18 @@
       </c>
       <c r="J406" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K406" s="5" t="n">
-        <v>12905600</v>
+        <v>12976500</v>
       </c>
       <c r="L406" s="5" t="n">
-        <v>31023</v>
+        <v>31194</v>
       </c>
       <c r="M406" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N406" s="3" t="inlineStr">
@@ -27056,18 +27056,18 @@
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K409" s="5" t="n">
-        <v>14762500</v>
+        <v>13997600</v>
       </c>
       <c r="L409" s="5" t="n">
-        <v>31210</v>
+        <v>29593</v>
       </c>
       <c r="M409" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N409" s="3" t="inlineStr">
@@ -27614,18 +27614,18 @@
       </c>
       <c r="J418" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K418" s="5" t="n">
-        <v>12829100</v>
+        <v>12899600</v>
       </c>
       <c r="L418" s="5" t="n">
-        <v>30839</v>
+        <v>31009</v>
       </c>
       <c r="M418" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N418" s="3" t="inlineStr">
@@ -27808,18 +27808,18 @@
       </c>
       <c r="J421" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K421" s="5" t="n">
-        <v>14675200</v>
+        <v>13914800</v>
       </c>
       <c r="L421" s="5" t="n">
-        <v>31026</v>
+        <v>29418</v>
       </c>
       <c r="M421" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N421" s="3" t="inlineStr">
@@ -28366,18 +28366,18 @@
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K430" s="5" t="n">
-        <v>12753600</v>
+        <v>12823700</v>
       </c>
       <c r="L430" s="5" t="n">
-        <v>30658</v>
+        <v>30826</v>
       </c>
       <c r="M430" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N430" s="3" t="inlineStr">
@@ -28560,18 +28560,18 @@
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K433" s="5" t="n">
-        <v>14588800</v>
+        <v>13832900</v>
       </c>
       <c r="L433" s="5" t="n">
-        <v>30843</v>
+        <v>29245</v>
       </c>
       <c r="M433" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N433" s="3" t="inlineStr">
@@ -29118,18 +29118,18 @@
       </c>
       <c r="J442" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K442" s="5" t="n">
-        <v>12678100</v>
+        <v>12747700</v>
       </c>
       <c r="L442" s="5" t="n">
-        <v>30476</v>
+        <v>30644</v>
       </c>
       <c r="M442" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N442" s="3" t="inlineStr">
@@ -29886,18 +29886,18 @@
       </c>
       <c r="J454" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K454" s="5" t="n">
-        <v>12639900</v>
+        <v>12709300</v>
       </c>
       <c r="L454" s="5" t="n">
-        <v>30384</v>
+        <v>30551</v>
       </c>
       <c r="M454" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N454" s="3" t="inlineStr">
@@ -30654,18 +30654,18 @@
       </c>
       <c r="J466" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K466" s="5" t="n">
-        <v>12602500</v>
+        <v>12671800</v>
       </c>
       <c r="L466" s="5" t="n">
-        <v>30294</v>
+        <v>30461</v>
       </c>
       <c r="M466" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N466" s="3" t="inlineStr">
@@ -31422,18 +31422,18 @@
       </c>
       <c r="J478" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K478" s="5" t="n">
-        <v>12564300</v>
+        <v>12633400</v>
       </c>
       <c r="L478" s="5" t="n">
-        <v>30203</v>
+        <v>30369</v>
       </c>
       <c r="M478" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N478" s="3" t="inlineStr">
@@ -32190,18 +32190,18 @@
       </c>
       <c r="J490" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K490" s="5" t="n">
-        <v>12527000</v>
+        <v>12595800</v>
       </c>
       <c r="L490" s="5" t="n">
-        <v>30113</v>
+        <v>30278</v>
       </c>
       <c r="M490" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N490" s="3" t="inlineStr">
@@ -32958,18 +32958,18 @@
       </c>
       <c r="J502" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K502" s="5" t="n">
-        <v>12527000</v>
+        <v>12595800</v>
       </c>
       <c r="L502" s="5" t="n">
-        <v>30113</v>
+        <v>30278</v>
       </c>
       <c r="M502" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N502" s="3" t="inlineStr">
@@ -33152,18 +33152,18 @@
       </c>
       <c r="J505" s="3" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K505" s="5" t="n">
-        <v>14886000</v>
+        <v>14114700</v>
       </c>
       <c r="L505" s="5" t="n">
-        <v>31471</v>
+        <v>29841</v>
       </c>
       <c r="M505" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N505" s="3" t="inlineStr">
@@ -33710,18 +33710,18 @@
       </c>
       <c r="J514" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K514" s="5" t="n">
-        <v>12488800</v>
+        <v>12557400</v>
       </c>
       <c r="L514" s="5" t="n">
-        <v>30021</v>
+        <v>30186</v>
       </c>
       <c r="M514" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N514" s="3" t="inlineStr">
@@ -33904,18 +33904,18 @@
       </c>
       <c r="J517" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K517" s="5" t="n">
-        <v>14284100</v>
+        <v>13544000</v>
       </c>
       <c r="L517" s="5" t="n">
-        <v>30199</v>
+        <v>28634</v>
       </c>
       <c r="M517" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N517" s="3" t="inlineStr">
@@ -34656,18 +34656,18 @@
       </c>
       <c r="J529" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K529" s="5" t="n">
-        <v>14241400</v>
+        <v>13503400</v>
       </c>
       <c r="L529" s="5" t="n">
-        <v>30109</v>
+        <v>28548</v>
       </c>
       <c r="M529" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N529" s="3" t="inlineStr">
@@ -35214,18 +35214,18 @@
       </c>
       <c r="J538" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K538" s="5" t="n">
-        <v>12413300</v>
+        <v>12481500</v>
       </c>
       <c r="L538" s="5" t="n">
-        <v>29840</v>
+        <v>30004</v>
       </c>
       <c r="M538" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N538" s="3" t="inlineStr">
@@ -35408,18 +35408,18 @@
       </c>
       <c r="J541" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K541" s="5" t="n">
-        <v>14197700</v>
+        <v>13462100</v>
       </c>
       <c r="L541" s="5" t="n">
-        <v>30016</v>
+        <v>28461</v>
       </c>
       <c r="M541" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N541" s="3" t="inlineStr">
@@ -35470,18 +35470,18 @@
       </c>
       <c r="J542" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.26%</t>
         </is>
       </c>
       <c r="K542" s="5" t="n">
-        <v>21438300</v>
+        <v>20356800</v>
       </c>
       <c r="L542" s="5" t="n">
-        <v>31620</v>
+        <v>30025</v>
       </c>
       <c r="M542" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N542" s="3" t="inlineStr">
@@ -35966,18 +35966,18 @@
       </c>
       <c r="J550" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K550" s="5" t="n">
-        <v>12375000</v>
+        <v>12443000</v>
       </c>
       <c r="L550" s="5" t="n">
-        <v>29748</v>
+        <v>29911</v>
       </c>
       <c r="M550" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N550" s="3" t="inlineStr">
@@ -36160,18 +36160,18 @@
       </c>
       <c r="J553" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K553" s="5" t="n">
-        <v>14154100</v>
+        <v>13420700</v>
       </c>
       <c r="L553" s="5" t="n">
-        <v>29924</v>
+        <v>28374</v>
       </c>
       <c r="M553" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N553" s="3" t="inlineStr">
@@ -36222,18 +36222,18 @@
       </c>
       <c r="J554" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.25%</t>
         </is>
       </c>
       <c r="K554" s="5" t="n">
-        <v>21373600</v>
+        <v>20299100</v>
       </c>
       <c r="L554" s="5" t="n">
-        <v>31524</v>
+        <v>29940</v>
       </c>
       <c r="M554" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N554" s="3" t="inlineStr">
@@ -36718,18 +36718,18 @@
       </c>
       <c r="J562" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K562" s="5" t="n">
-        <v>12299500</v>
+        <v>12367100</v>
       </c>
       <c r="L562" s="5" t="n">
-        <v>29566</v>
+        <v>29729</v>
       </c>
       <c r="M562" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N562" s="3" t="inlineStr">
@@ -36773,25 +36773,25 @@
         </is>
       </c>
       <c r="H563" s="5" t="n">
-        <v>1902700019312000</v>
+        <v>19312000</v>
       </c>
       <c r="I563" s="5" t="n">
-        <v>3124302166358</v>
+        <v>31711</v>
       </c>
       <c r="J563" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K563" s="5" t="n">
-        <v>1758071034093900</v>
+        <v>17007700</v>
       </c>
       <c r="L563" s="5" t="n">
-        <v>2886816147937</v>
+        <v>27927</v>
       </c>
       <c r="M563" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N563" s="3" t="inlineStr">
@@ -36912,18 +36912,18 @@
       </c>
       <c r="J565" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K565" s="5" t="n">
-        <v>14066800</v>
+        <v>13337900</v>
       </c>
       <c r="L565" s="5" t="n">
-        <v>29740</v>
+        <v>28199</v>
       </c>
       <c r="M565" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N565" s="3" t="inlineStr">
@@ -36974,18 +36974,18 @@
       </c>
       <c r="J566" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.21%</t>
         </is>
       </c>
       <c r="K566" s="5" t="n">
-        <v>21244200</v>
+        <v>20183800</v>
       </c>
       <c r="L566" s="5" t="n">
-        <v>31334</v>
+        <v>29770</v>
       </c>
       <c r="M566" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N566" s="3" t="inlineStr">
@@ -37470,18 +37470,18 @@
       </c>
       <c r="J574" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K574" s="5" t="n">
-        <v>12224000</v>
+        <v>12291100</v>
       </c>
       <c r="L574" s="5" t="n">
-        <v>29385</v>
+        <v>29546</v>
       </c>
       <c r="M574" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N574" s="3" t="inlineStr">
@@ -37525,25 +37525,25 @@
         </is>
       </c>
       <c r="H575" s="5" t="n">
-        <v>1891000019194000</v>
+        <v>19194000</v>
       </c>
       <c r="I575" s="5" t="n">
-        <v>3105090343504</v>
+        <v>31517</v>
       </c>
       <c r="J575" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K575" s="5" t="n">
-        <v>1747260380235000</v>
+        <v>16903900</v>
       </c>
       <c r="L575" s="5" t="n">
-        <v>2869064663768</v>
+        <v>27757</v>
       </c>
       <c r="M575" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N575" s="3" t="inlineStr">
@@ -37664,18 +37664,18 @@
       </c>
       <c r="J577" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K577" s="5" t="n">
-        <v>13980400</v>
+        <v>13256000</v>
       </c>
       <c r="L577" s="5" t="n">
-        <v>29557</v>
+        <v>28025</v>
       </c>
       <c r="M577" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N577" s="3" t="inlineStr">
@@ -37726,18 +37726,18 @@
       </c>
       <c r="J578" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.18%</t>
         </is>
       </c>
       <c r="K578" s="5" t="n">
-        <v>21114800</v>
+        <v>20068500</v>
       </c>
       <c r="L578" s="5" t="n">
-        <v>31143</v>
+        <v>29600</v>
       </c>
       <c r="M578" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N578" s="3" t="inlineStr">
@@ -38153,25 +38153,25 @@
         </is>
       </c>
       <c r="H585" s="5" t="n">
-        <v>1757200017836000</v>
+        <v>17836000</v>
       </c>
       <c r="I585" s="5" t="n">
-        <v>3115602868504</v>
+        <v>31624</v>
       </c>
       <c r="J585" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K585" s="5" t="n">
-        <v>1623630851480200</v>
+        <v>15707900</v>
       </c>
       <c r="L585" s="5" t="n">
-        <v>2878778105461</v>
+        <v>27851</v>
       </c>
       <c r="M585" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N585" s="3" t="inlineStr">
@@ -38222,18 +38222,18 @@
       </c>
       <c r="J586" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K586" s="5" t="n">
-        <v>12148500</v>
+        <v>12215200</v>
       </c>
       <c r="L586" s="5" t="n">
-        <v>29203</v>
+        <v>29363</v>
       </c>
       <c r="M586" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N586" s="3" t="inlineStr">
@@ -38277,25 +38277,25 @@
         </is>
       </c>
       <c r="H587" s="5" t="n">
-        <v>1879400019076000</v>
+        <v>19076000</v>
       </c>
       <c r="I587" s="5" t="n">
-        <v>3086042724263</v>
+        <v>31323</v>
       </c>
       <c r="J587" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K587" s="5" t="n">
-        <v>1736542125125900</v>
+        <v>16799900</v>
       </c>
       <c r="L587" s="5" t="n">
-        <v>2851464901685</v>
+        <v>27586</v>
       </c>
       <c r="M587" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N587" s="3" t="inlineStr">
@@ -38416,18 +38416,18 @@
       </c>
       <c r="J589" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K589" s="5" t="n">
-        <v>13893100</v>
+        <v>13173200</v>
       </c>
       <c r="L589" s="5" t="n">
-        <v>29372</v>
+        <v>27850</v>
       </c>
       <c r="M589" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N589" s="3" t="inlineStr">
@@ -38478,18 +38478,18 @@
       </c>
       <c r="J590" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="K590" s="5" t="n">
-        <v>20985500</v>
+        <v>19953200</v>
       </c>
       <c r="L590" s="5" t="n">
-        <v>30952</v>
+        <v>29429</v>
       </c>
       <c r="M590" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N590" s="3" t="inlineStr">
@@ -38905,25 +38905,25 @@
         </is>
       </c>
       <c r="H597" s="5" t="n">
-        <v>1757200017836000</v>
+        <v>17836000</v>
       </c>
       <c r="I597" s="5" t="n">
-        <v>3115602868504</v>
+        <v>31624</v>
       </c>
       <c r="J597" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K597" s="5" t="n">
-        <v>1623630851480200</v>
+        <v>15707900</v>
       </c>
       <c r="L597" s="5" t="n">
-        <v>2878778105461</v>
+        <v>27851</v>
       </c>
       <c r="M597" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N597" s="3" t="inlineStr">
@@ -38974,18 +38974,18 @@
       </c>
       <c r="J598" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K598" s="5" t="n">
-        <v>12148500</v>
+        <v>12215200</v>
       </c>
       <c r="L598" s="5" t="n">
-        <v>29203</v>
+        <v>29363</v>
       </c>
       <c r="M598" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N598" s="3" t="inlineStr">
@@ -39029,25 +39029,25 @@
         </is>
       </c>
       <c r="H599" s="5" t="n">
-        <v>1879400019076000</v>
+        <v>19076000</v>
       </c>
       <c r="I599" s="5" t="n">
-        <v>3086042724263</v>
+        <v>31323</v>
       </c>
       <c r="J599" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K599" s="5" t="n">
-        <v>1736542125125900</v>
+        <v>16799900</v>
       </c>
       <c r="L599" s="5" t="n">
-        <v>2851464901685</v>
+        <v>27586</v>
       </c>
       <c r="M599" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N599" s="3" t="inlineStr">
@@ -39168,18 +39168,18 @@
       </c>
       <c r="J601" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K601" s="5" t="n">
-        <v>13893100</v>
+        <v>13173200</v>
       </c>
       <c r="L601" s="5" t="n">
-        <v>29372</v>
+        <v>27850</v>
       </c>
       <c r="M601" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N601" s="3" t="inlineStr">
@@ -39230,18 +39230,18 @@
       </c>
       <c r="J602" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.15%</t>
         </is>
       </c>
       <c r="K602" s="5" t="n">
-        <v>20985500</v>
+        <v>19953200</v>
       </c>
       <c r="L602" s="5" t="n">
-        <v>30952</v>
+        <v>29429</v>
       </c>
       <c r="M602" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N602" s="3" t="inlineStr">
@@ -39657,25 +39657,25 @@
         </is>
       </c>
       <c r="H609" s="5" t="n">
-        <v>1746400017726000</v>
+        <v>17726000</v>
       </c>
       <c r="I609" s="5" t="n">
-        <v>3096453932138</v>
+        <v>31429</v>
       </c>
       <c r="J609" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K609" s="5" t="n">
-        <v>1613651786378500</v>
+        <v>15610900</v>
       </c>
       <c r="L609" s="5" t="n">
-        <v>2861084727621</v>
+        <v>27679</v>
       </c>
       <c r="M609" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N609" s="3" t="inlineStr">
@@ -39726,18 +39726,18 @@
       </c>
       <c r="J610" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K610" s="5" t="n">
-        <v>12072900</v>
+        <v>12139300</v>
       </c>
       <c r="L610" s="5" t="n">
-        <v>29021</v>
+        <v>29181</v>
       </c>
       <c r="M610" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N610" s="3" t="inlineStr">
@@ -39781,25 +39781,25 @@
         </is>
       </c>
       <c r="H611" s="5" t="n">
-        <v>1867800018958000</v>
+        <v>18958000</v>
       </c>
       <c r="I611" s="5" t="n">
-        <v>3066995105021</v>
+        <v>31130</v>
       </c>
       <c r="J611" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K611" s="5" t="n">
-        <v>1725823870016800</v>
+        <v>16696000</v>
       </c>
       <c r="L611" s="5" t="n">
-        <v>2833865139601</v>
+        <v>27415</v>
       </c>
       <c r="M611" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N611" s="3" t="inlineStr">
@@ -39920,18 +39920,18 @@
       </c>
       <c r="J613" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K613" s="5" t="n">
-        <v>13806700</v>
+        <v>13091300</v>
       </c>
       <c r="L613" s="5" t="n">
-        <v>29190</v>
+        <v>27677</v>
       </c>
       <c r="M613" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N613" s="3" t="inlineStr">
@@ -39982,18 +39982,18 @@
       </c>
       <c r="J614" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>12.11%</t>
         </is>
       </c>
       <c r="K614" s="5" t="n">
-        <v>20856100</v>
+        <v>19837900</v>
       </c>
       <c r="L614" s="5" t="n">
-        <v>30761</v>
+        <v>29259</v>
       </c>
       <c r="M614" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N614" s="3" t="inlineStr">
@@ -40409,25 +40409,25 @@
         </is>
       </c>
       <c r="H621" s="5" t="n">
-        <v>1735600017616000</v>
+        <v>17616000</v>
       </c>
       <c r="I621" s="5" t="n">
-        <v>3077304995773</v>
+        <v>31234</v>
       </c>
       <c r="J621" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K621" s="5" t="n">
-        <v>1603672721276900</v>
+        <v>15514100</v>
       </c>
       <c r="L621" s="5" t="n">
-        <v>2843391349782</v>
+        <v>27507</v>
       </c>
       <c r="M621" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N621" s="3" t="inlineStr">
@@ -40478,18 +40478,18 @@
       </c>
       <c r="J622" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K622" s="5" t="n">
-        <v>11996500</v>
+        <v>12062400</v>
       </c>
       <c r="L622" s="5" t="n">
-        <v>28838</v>
+        <v>28996</v>
       </c>
       <c r="M622" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N622" s="3" t="inlineStr">
@@ -40533,25 +40533,25 @@
         </is>
       </c>
       <c r="H623" s="5" t="n">
-        <v>1856100018839000</v>
+        <v>18839000</v>
       </c>
       <c r="I623" s="5" t="n">
-        <v>3047783282166</v>
+        <v>30934</v>
       </c>
       <c r="J623" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K623" s="5" t="n">
-        <v>1715013216156900</v>
+        <v>16591100</v>
       </c>
       <c r="L623" s="5" t="n">
-        <v>2816113655430</v>
+        <v>27243</v>
       </c>
       <c r="M623" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N623" s="3" t="inlineStr">
@@ -40672,18 +40672,18 @@
       </c>
       <c r="J625" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K625" s="5" t="n">
-        <v>13719400</v>
+        <v>13008500</v>
       </c>
       <c r="L625" s="5" t="n">
-        <v>29005</v>
+        <v>27502</v>
       </c>
       <c r="M625" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N625" s="3" t="inlineStr">
@@ -40734,18 +40734,18 @@
       </c>
       <c r="J626" s="3" t="inlineStr">
         <is>
-          <t>7.58%</t>
+          <t>12.08%</t>
         </is>
       </c>
       <c r="K626" s="5" t="n">
-        <v>20732100</v>
+        <v>19722600</v>
       </c>
       <c r="L626" s="5" t="n">
-        <v>30578</v>
+        <v>29089</v>
       </c>
       <c r="M626" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N626" s="3" t="inlineStr">
@@ -41161,25 +41161,25 @@
         </is>
       </c>
       <c r="H633" s="5" t="n">
-        <v>1724800017507000</v>
+        <v>17507000</v>
       </c>
       <c r="I633" s="5" t="n">
-        <v>3058156059410</v>
+        <v>31041</v>
       </c>
       <c r="J633" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K633" s="5" t="n">
-        <v>1593693656176100</v>
+        <v>15418100</v>
       </c>
       <c r="L633" s="5" t="n">
-        <v>2825697971943</v>
+        <v>27337</v>
       </c>
       <c r="M633" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N633" s="3" t="inlineStr">
@@ -41230,18 +41230,18 @@
       </c>
       <c r="J634" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K634" s="5" t="n">
-        <v>11921000</v>
+        <v>11986500</v>
       </c>
       <c r="L634" s="5" t="n">
-        <v>28656</v>
+        <v>28814</v>
       </c>
       <c r="M634" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N634" s="3" t="inlineStr">
@@ -41285,25 +41285,25 @@
         </is>
       </c>
       <c r="H635" s="5" t="n">
-        <v>1844500018722000</v>
+        <v>18722000</v>
       </c>
       <c r="I635" s="5" t="n">
-        <v>3028735662926</v>
+        <v>30742</v>
       </c>
       <c r="J635" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K635" s="5" t="n">
-        <v>1704294961048800</v>
+        <v>16488200</v>
       </c>
       <c r="L635" s="5" t="n">
-        <v>2798513893348</v>
+        <v>27074</v>
       </c>
       <c r="M635" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N635" s="3" t="inlineStr">
@@ -41424,18 +41424,18 @@
       </c>
       <c r="J637" s="3" t="inlineStr">
         <is>
-          <t>7.12%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K637" s="5" t="n">
-        <v>13633000</v>
+        <v>12926600</v>
       </c>
       <c r="L637" s="5" t="n">
-        <v>28822</v>
+        <v>27329</v>
       </c>
       <c r="M637" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N637" s="3" t="inlineStr">
@@ -41486,18 +41486,18 @@
       </c>
       <c r="J638" s="3" t="inlineStr">
         <is>
-          <t>7.54%</t>
+          <t>12.04%</t>
         </is>
       </c>
       <c r="K638" s="5" t="n">
-        <v>20610500</v>
+        <v>19607300</v>
       </c>
       <c r="L638" s="5" t="n">
-        <v>30399</v>
+        <v>28919</v>
       </c>
       <c r="M638" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N638" s="3" t="inlineStr">
@@ -41913,25 +41913,25 @@
         </is>
       </c>
       <c r="H645" s="5" t="n">
-        <v>1708600017342000</v>
+        <v>17342000</v>
       </c>
       <c r="I645" s="5" t="n">
-        <v>3029432654862</v>
+        <v>30748</v>
       </c>
       <c r="J645" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K645" s="5" t="n">
-        <v>1578725058523700</v>
+        <v>15272800</v>
       </c>
       <c r="L645" s="5" t="n">
-        <v>2799157905184</v>
+        <v>27079</v>
       </c>
       <c r="M645" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N645" s="3" t="inlineStr">
@@ -41982,18 +41982,18 @@
       </c>
       <c r="J646" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K646" s="5" t="n">
-        <v>11807200</v>
+        <v>11872100</v>
       </c>
       <c r="L646" s="5" t="n">
-        <v>28383</v>
+        <v>28539</v>
       </c>
       <c r="M646" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N646" s="3" t="inlineStr">
@@ -42037,25 +42037,25 @@
         </is>
       </c>
       <c r="H647" s="5" t="n">
-        <v>1827000018544000</v>
+        <v>18544000</v>
       </c>
       <c r="I647" s="5" t="n">
-        <v>3000000030450</v>
+        <v>30450</v>
       </c>
       <c r="J647" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K647" s="5" t="n">
-        <v>1688125179634300</v>
+        <v>16331400</v>
       </c>
       <c r="L647" s="5" t="n">
-        <v>2771962528135</v>
+        <v>26817</v>
       </c>
       <c r="M647" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N647" s="3" t="inlineStr">
@@ -42681,25 +42681,25 @@
         </is>
       </c>
       <c r="H657" s="5" t="n">
-        <v>1686900017122000</v>
+        <v>17122000</v>
       </c>
       <c r="I657" s="5" t="n">
-        <v>2990957477167</v>
+        <v>30358</v>
       </c>
       <c r="J657" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K657" s="5" t="n">
-        <v>1558674529570400</v>
+        <v>15079100</v>
       </c>
       <c r="L657" s="5" t="n">
-        <v>2763607321933</v>
+        <v>26736</v>
       </c>
       <c r="M657" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N657" s="3" t="inlineStr">
@@ -42750,18 +42750,18 @@
       </c>
       <c r="J658" s="3" t="inlineStr">
         <is>
-          <t>9.00%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K658" s="5" t="n">
-        <v>11656100</v>
+        <v>11720200</v>
       </c>
       <c r="L658" s="5" t="n">
-        <v>28019</v>
+        <v>28174</v>
       </c>
       <c r="M658" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減9.0%)</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N658" s="3" t="inlineStr">
@@ -42805,25 +42805,25 @@
         </is>
       </c>
       <c r="H659" s="5" t="n">
-        <v>1803700018308000</v>
+        <v>18308000</v>
       </c>
       <c r="I659" s="5" t="n">
-        <v>2961740588355</v>
+        <v>30062</v>
       </c>
       <c r="J659" s="3" t="inlineStr">
         <is>
-          <t>7.60%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K659" s="5" t="n">
-        <v>1666596270666300</v>
+        <v>16123600</v>
       </c>
       <c r="L659" s="5" t="n">
-        <v>2736611281882</v>
+        <v>26476</v>
       </c>
       <c r="M659" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減3.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N659" s="3" t="inlineStr">
@@ -53137,8 +53137,8 @@
       <c r="E25" s="23" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$190270001931万
-$3,124,302,166,358/呎
+$1931万
+$31,711/呎
 (在售)</t>
         </is>
       </c>
@@ -53240,8 +53240,8 @@
       <c r="E26" s="23" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$189100001919万
-$3,105,090,343,504/呎
+$1919万
+$31,517/呎
 (在售)</t>
         </is>
       </c>
@@ -53343,8 +53343,8 @@
       <c r="E27" s="23" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$187940001908万
-$3,086,042,724,263/呎
+$1908万
+$31,323/呎
 (在售)</t>
         </is>
       </c>
@@ -53359,8 +53359,8 @@
       <c r="G27" s="23" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$175720001784万
-$3,115,602,868,504/呎
+$1784万
+$31,624/呎
 (在售)</t>
         </is>
       </c>
@@ -53446,8 +53446,8 @@
       <c r="E28" s="24" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$187940001908万
-$3,086,042,724,263/呎
+$1908万
+$31,323/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53462,8 +53462,8 @@
       <c r="G28" s="24" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$175720001784万
-$3,115,602,868,504/呎
+$1784万
+$31,624/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53549,8 +53549,8 @@
       <c r="E29" s="24" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$186780001896万
-$3,066,995,105,021/呎
+$1896万
+$31,130/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53565,8 +53565,8 @@
       <c r="G29" s="24" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$174640001773万
-$3,096,453,932,138/呎
+$1773万
+$31,429/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53652,8 +53652,8 @@
       <c r="E30" s="23" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$185610001884万
-$3,047,783,282,166/呎
+$1884万
+$30,934/呎
 (在售)</t>
         </is>
       </c>
@@ -53668,8 +53668,8 @@
       <c r="G30" s="23" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$173560001762万
-$3,077,304,995,773/呎
+$1762万
+$31,234/呎
 (在售)</t>
         </is>
       </c>
@@ -53755,8 +53755,8 @@
       <c r="E31" s="23" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$184450001872万
-$3,028,735,662,926/呎
+$1872万
+$30,742/呎
 (在售)</t>
         </is>
       </c>
@@ -53771,8 +53771,8 @@
       <c r="G31" s="23" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$172480001751万
-$3,058,156,059,410/呎
+$1751万
+$31,041/呎
 (在售)</t>
         </is>
       </c>
@@ -53858,8 +53858,8 @@
       <c r="E32" s="24" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$182700001854万
-$3,000,000,030,450/呎
+$1854万
+$30,450/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53874,8 +53874,8 @@
       <c r="G32" s="24" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$170860001734万
-$3,029,432,654,862/呎
+$1734万
+$30,748/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53961,8 +53961,8 @@
       <c r="E33" s="24" t="inlineStr">
         <is>
           <t>D | 609呎 (2房)
-$180370001831万
-$2,961,740,588,355/呎
+$1831万
+$30,062/呎
 (已定价未售)</t>
         </is>
       </c>
@@ -53977,8 +53977,8 @@
       <c r="G33" s="24" t="inlineStr">
         <is>
           <t>F | 564呎 (2房)
-$168690001712万
-$2,990,957,477,167/呎
+$1712万
+$30,358/呎
 (已定价未售)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
revert: remove sorting dropdown from web interface
</commit_message>
<xml_diff>
--- a/files/九龙-启德-Henley Park.xlsx
+++ b/files/九龙-启德-Henley Park.xlsx
@@ -22318,18 +22318,18 @@
       </c>
       <c r="J334" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K334" s="5" t="n">
-        <v>13509000</v>
+        <v>13509060</v>
       </c>
       <c r="L334" s="5" t="n">
         <v>32474</v>
       </c>
       <c r="M334" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N334" s="3" t="inlineStr">
@@ -23086,18 +23086,18 @@
       </c>
       <c r="J346" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K346" s="5" t="n">
-        <v>13356200</v>
+        <v>13356255</v>
       </c>
       <c r="L346" s="5" t="n">
         <v>32106</v>
       </c>
       <c r="M346" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N346" s="3" t="inlineStr">
@@ -23846,18 +23846,18 @@
       </c>
       <c r="J358" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K358" s="5" t="n">
-        <v>13280300</v>
+        <v>13280310</v>
       </c>
       <c r="L358" s="5" t="n">
         <v>31924</v>
       </c>
       <c r="M358" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N358" s="3" t="inlineStr">
@@ -24606,18 +24606,18 @@
       </c>
       <c r="J370" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K370" s="5" t="n">
-        <v>13204300</v>
+        <v>13204365</v>
       </c>
       <c r="L370" s="5" t="n">
         <v>31741</v>
       </c>
       <c r="M370" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N370" s="3" t="inlineStr">
@@ -25358,18 +25358,18 @@
       </c>
       <c r="J382" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K382" s="5" t="n">
-        <v>13128400</v>
+        <v>13128420</v>
       </c>
       <c r="L382" s="5" t="n">
         <v>31559</v>
       </c>
       <c r="M382" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N382" s="3" t="inlineStr">
@@ -26110,18 +26110,18 @@
       </c>
       <c r="J394" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K394" s="5" t="n">
-        <v>13052400</v>
+        <v>13052475</v>
       </c>
       <c r="L394" s="5" t="n">
         <v>31376</v>
       </c>
       <c r="M394" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N394" s="3" t="inlineStr">
@@ -26862,18 +26862,18 @@
       </c>
       <c r="J406" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K406" s="5" t="n">
-        <v>12976500</v>
+        <v>12976530</v>
       </c>
       <c r="L406" s="5" t="n">
         <v>31194</v>
       </c>
       <c r="M406" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N406" s="3" t="inlineStr">
@@ -27056,18 +27056,18 @@
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K409" s="5" t="n">
-        <v>13997600</v>
+        <v>14543010</v>
       </c>
       <c r="L409" s="5" t="n">
-        <v>29593</v>
+        <v>30746</v>
       </c>
       <c r="M409" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N409" s="3" t="inlineStr">
@@ -27614,18 +27614,18 @@
       </c>
       <c r="J418" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K418" s="5" t="n">
-        <v>12899600</v>
+        <v>12899670</v>
       </c>
       <c r="L418" s="5" t="n">
         <v>31009</v>
       </c>
       <c r="M418" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N418" s="3" t="inlineStr">
@@ -27808,18 +27808,18 @@
       </c>
       <c r="J421" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K421" s="5" t="n">
-        <v>13914800</v>
+        <v>14457000</v>
       </c>
       <c r="L421" s="5" t="n">
-        <v>29418</v>
+        <v>30564</v>
       </c>
       <c r="M421" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N421" s="3" t="inlineStr">
@@ -28366,18 +28366,18 @@
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K430" s="5" t="n">
-        <v>12823700</v>
+        <v>12823725</v>
       </c>
       <c r="L430" s="5" t="n">
         <v>30826</v>
       </c>
       <c r="M430" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N430" s="3" t="inlineStr">
@@ -28560,18 +28560,18 @@
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K433" s="5" t="n">
-        <v>13832900</v>
+        <v>14371905</v>
       </c>
       <c r="L433" s="5" t="n">
-        <v>29245</v>
+        <v>30385</v>
       </c>
       <c r="M433" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N433" s="3" t="inlineStr">
@@ -29118,18 +29118,18 @@
       </c>
       <c r="J442" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K442" s="5" t="n">
-        <v>12747700</v>
+        <v>12747780</v>
       </c>
       <c r="L442" s="5" t="n">
         <v>30644</v>
       </c>
       <c r="M442" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N442" s="3" t="inlineStr">
@@ -29886,18 +29886,18 @@
       </c>
       <c r="J454" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K454" s="5" t="n">
-        <v>12709300</v>
+        <v>12709350</v>
       </c>
       <c r="L454" s="5" t="n">
         <v>30551</v>
       </c>
       <c r="M454" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N454" s="3" t="inlineStr">
@@ -30654,18 +30654,18 @@
       </c>
       <c r="J466" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K466" s="5" t="n">
-        <v>12671800</v>
+        <v>12671835</v>
       </c>
       <c r="L466" s="5" t="n">
         <v>30461</v>
       </c>
       <c r="M466" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N466" s="3" t="inlineStr">
@@ -31422,18 +31422,18 @@
       </c>
       <c r="J478" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K478" s="5" t="n">
-        <v>12633400</v>
+        <v>12633405</v>
       </c>
       <c r="L478" s="5" t="n">
         <v>30369</v>
       </c>
       <c r="M478" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N478" s="3" t="inlineStr">
@@ -32190,18 +32190,18 @@
       </c>
       <c r="J490" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K490" s="5" t="n">
-        <v>12595800</v>
+        <v>12595890</v>
       </c>
       <c r="L490" s="5" t="n">
-        <v>30278</v>
+        <v>30279</v>
       </c>
       <c r="M490" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N490" s="3" t="inlineStr">
@@ -32958,18 +32958,18 @@
       </c>
       <c r="J502" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K502" s="5" t="n">
-        <v>12595800</v>
+        <v>12595890</v>
       </c>
       <c r="L502" s="5" t="n">
-        <v>30278</v>
+        <v>30279</v>
       </c>
       <c r="M502" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N502" s="3" t="inlineStr">
@@ -33152,18 +33152,18 @@
       </c>
       <c r="J505" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K505" s="5" t="n">
-        <v>14114700</v>
+        <v>14114790</v>
       </c>
       <c r="L505" s="5" t="n">
         <v>29841</v>
       </c>
       <c r="M505" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N505" s="3" t="inlineStr">
@@ -33710,18 +33710,18 @@
       </c>
       <c r="J514" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K514" s="5" t="n">
-        <v>12557400</v>
+        <v>12557460</v>
       </c>
       <c r="L514" s="5" t="n">
         <v>30186</v>
       </c>
       <c r="M514" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N514" s="3" t="inlineStr">
@@ -33904,18 +33904,18 @@
       </c>
       <c r="J517" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K517" s="5" t="n">
-        <v>13544000</v>
+        <v>14071785</v>
       </c>
       <c r="L517" s="5" t="n">
-        <v>28634</v>
+        <v>29750</v>
       </c>
       <c r="M517" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N517" s="3" t="inlineStr">
@@ -34656,18 +34656,18 @@
       </c>
       <c r="J529" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K529" s="5" t="n">
-        <v>13503400</v>
+        <v>14029695</v>
       </c>
       <c r="L529" s="5" t="n">
-        <v>28548</v>
+        <v>29661</v>
       </c>
       <c r="M529" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N529" s="3" t="inlineStr">
@@ -35214,18 +35214,18 @@
       </c>
       <c r="J538" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K538" s="5" t="n">
-        <v>12481500</v>
+        <v>12481515</v>
       </c>
       <c r="L538" s="5" t="n">
         <v>30004</v>
       </c>
       <c r="M538" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N538" s="3" t="inlineStr">
@@ -35408,18 +35408,18 @@
       </c>
       <c r="J541" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K541" s="5" t="n">
-        <v>13462100</v>
+        <v>13986690</v>
       </c>
       <c r="L541" s="5" t="n">
-        <v>28461</v>
+        <v>29570</v>
       </c>
       <c r="M541" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N541" s="3" t="inlineStr">
@@ -35966,18 +35966,18 @@
       </c>
       <c r="J550" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K550" s="5" t="n">
-        <v>12443000</v>
+        <v>12443085</v>
       </c>
       <c r="L550" s="5" t="n">
         <v>29911</v>
       </c>
       <c r="M550" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N550" s="3" t="inlineStr">
@@ -36160,18 +36160,18 @@
       </c>
       <c r="J553" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K553" s="5" t="n">
-        <v>13420700</v>
+        <v>13943685</v>
       </c>
       <c r="L553" s="5" t="n">
-        <v>28374</v>
+        <v>29479</v>
       </c>
       <c r="M553" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N553" s="3" t="inlineStr">
@@ -36718,18 +36718,18 @@
       </c>
       <c r="J562" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K562" s="5" t="n">
-        <v>12367100</v>
+        <v>12367140</v>
       </c>
       <c r="L562" s="5" t="n">
         <v>29729</v>
       </c>
       <c r="M562" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N562" s="3" t="inlineStr">
@@ -36912,18 +36912,18 @@
       </c>
       <c r="J565" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K565" s="5" t="n">
-        <v>13337900</v>
+        <v>13857675</v>
       </c>
       <c r="L565" s="5" t="n">
-        <v>28199</v>
+        <v>29297</v>
       </c>
       <c r="M565" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N565" s="3" t="inlineStr">
@@ -37470,18 +37470,18 @@
       </c>
       <c r="J574" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K574" s="5" t="n">
-        <v>12291100</v>
+        <v>12291195</v>
       </c>
       <c r="L574" s="5" t="n">
         <v>29546</v>
       </c>
       <c r="M574" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N574" s="3" t="inlineStr">
@@ -37664,18 +37664,18 @@
       </c>
       <c r="J577" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K577" s="5" t="n">
-        <v>13256000</v>
+        <v>13772580</v>
       </c>
       <c r="L577" s="5" t="n">
-        <v>28025</v>
+        <v>29118</v>
       </c>
       <c r="M577" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N577" s="3" t="inlineStr">
@@ -38222,18 +38222,18 @@
       </c>
       <c r="J586" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K586" s="5" t="n">
-        <v>12215200</v>
+        <v>12215250</v>
       </c>
       <c r="L586" s="5" t="n">
-        <v>29363</v>
+        <v>29364</v>
       </c>
       <c r="M586" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N586" s="3" t="inlineStr">
@@ -38416,18 +38416,18 @@
       </c>
       <c r="J589" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K589" s="5" t="n">
-        <v>13173200</v>
+        <v>13686570</v>
       </c>
       <c r="L589" s="5" t="n">
-        <v>27850</v>
+        <v>28936</v>
       </c>
       <c r="M589" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N589" s="3" t="inlineStr">
@@ -38974,18 +38974,18 @@
       </c>
       <c r="J598" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K598" s="5" t="n">
-        <v>12215200</v>
+        <v>12215250</v>
       </c>
       <c r="L598" s="5" t="n">
-        <v>29363</v>
+        <v>29364</v>
       </c>
       <c r="M598" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N598" s="3" t="inlineStr">
@@ -39168,18 +39168,18 @@
       </c>
       <c r="J601" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K601" s="5" t="n">
-        <v>13173200</v>
+        <v>13686570</v>
       </c>
       <c r="L601" s="5" t="n">
-        <v>27850</v>
+        <v>28936</v>
       </c>
       <c r="M601" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N601" s="3" t="inlineStr">
@@ -39726,18 +39726,18 @@
       </c>
       <c r="J610" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K610" s="5" t="n">
-        <v>12139300</v>
+        <v>12139305</v>
       </c>
       <c r="L610" s="5" t="n">
         <v>29181</v>
       </c>
       <c r="M610" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N610" s="3" t="inlineStr">
@@ -39920,18 +39920,18 @@
       </c>
       <c r="J613" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K613" s="5" t="n">
-        <v>13091300</v>
+        <v>13601475</v>
       </c>
       <c r="L613" s="5" t="n">
-        <v>27677</v>
+        <v>28756</v>
       </c>
       <c r="M613" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N613" s="3" t="inlineStr">
@@ -40478,18 +40478,18 @@
       </c>
       <c r="J622" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K622" s="5" t="n">
-        <v>12062400</v>
+        <v>12062445</v>
       </c>
       <c r="L622" s="5" t="n">
         <v>28996</v>
       </c>
       <c r="M622" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N622" s="3" t="inlineStr">
@@ -40672,18 +40672,18 @@
       </c>
       <c r="J625" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K625" s="5" t="n">
-        <v>13008500</v>
+        <v>13515465</v>
       </c>
       <c r="L625" s="5" t="n">
-        <v>27502</v>
+        <v>28574</v>
       </c>
       <c r="M625" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N625" s="3" t="inlineStr">
@@ -41230,7 +41230,7 @@
       </c>
       <c r="J634" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K634" s="5" t="n">
@@ -41241,7 +41241,7 @@
       </c>
       <c r="M634" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N634" s="3" t="inlineStr">
@@ -41424,18 +41424,18 @@
       </c>
       <c r="J637" s="3" t="inlineStr">
         <is>
-          <t>11.93%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K637" s="5" t="n">
-        <v>12926600</v>
+        <v>13430370</v>
       </c>
       <c r="L637" s="5" t="n">
-        <v>27329</v>
+        <v>28394</v>
       </c>
       <c r="M637" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N637" s="3" t="inlineStr">
@@ -41982,18 +41982,18 @@
       </c>
       <c r="J646" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K646" s="5" t="n">
-        <v>11872100</v>
+        <v>11872125</v>
       </c>
       <c r="L646" s="5" t="n">
         <v>28539</v>
       </c>
       <c r="M646" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N646" s="3" t="inlineStr">
@@ -42750,18 +42750,18 @@
       </c>
       <c r="J658" s="3" t="inlineStr">
         <is>
-          <t>8.50%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="K658" s="5" t="n">
-        <v>11720200</v>
+        <v>11720235</v>
       </c>
       <c r="L658" s="5" t="n">
         <v>28174</v>
       </c>
       <c r="M658" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 (減8.5%)</t>
+          <t>現金付款計劃 - 90天成交</t>
         </is>
       </c>
       <c r="N658" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix: correct target units high-precision discount calculation
</commit_message>
<xml_diff>
--- a/files/九龙-启德-Henley Park.xlsx
+++ b/files/九龙-启德-Henley Park.xlsx
@@ -22318,18 +22318,18 @@
       </c>
       <c r="J334" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K334" s="5" t="n">
-        <v>13509060</v>
+        <v>13509000</v>
       </c>
       <c r="L334" s="5" t="n">
         <v>32474</v>
       </c>
       <c r="M334" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N334" s="3" t="inlineStr">
@@ -23086,18 +23086,18 @@
       </c>
       <c r="J346" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K346" s="5" t="n">
-        <v>13356255</v>
+        <v>13356200</v>
       </c>
       <c r="L346" s="5" t="n">
         <v>32106</v>
       </c>
       <c r="M346" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N346" s="3" t="inlineStr">
@@ -23846,18 +23846,18 @@
       </c>
       <c r="J358" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K358" s="5" t="n">
-        <v>13280310</v>
+        <v>13280300</v>
       </c>
       <c r="L358" s="5" t="n">
         <v>31924</v>
       </c>
       <c r="M358" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N358" s="3" t="inlineStr">
@@ -24606,18 +24606,18 @@
       </c>
       <c r="J370" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K370" s="5" t="n">
-        <v>13204365</v>
+        <v>13204300</v>
       </c>
       <c r="L370" s="5" t="n">
         <v>31741</v>
       </c>
       <c r="M370" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N370" s="3" t="inlineStr">
@@ -25358,18 +25358,18 @@
       </c>
       <c r="J382" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K382" s="5" t="n">
-        <v>13128420</v>
+        <v>13128400</v>
       </c>
       <c r="L382" s="5" t="n">
         <v>31559</v>
       </c>
       <c r="M382" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N382" s="3" t="inlineStr">
@@ -26110,18 +26110,18 @@
       </c>
       <c r="J394" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K394" s="5" t="n">
-        <v>13052475</v>
+        <v>13052400</v>
       </c>
       <c r="L394" s="5" t="n">
         <v>31376</v>
       </c>
       <c r="M394" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N394" s="3" t="inlineStr">
@@ -26862,18 +26862,18 @@
       </c>
       <c r="J406" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K406" s="5" t="n">
-        <v>12976530</v>
+        <v>12976500</v>
       </c>
       <c r="L406" s="5" t="n">
         <v>31194</v>
       </c>
       <c r="M406" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N406" s="3" t="inlineStr">
@@ -27056,18 +27056,18 @@
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K409" s="5" t="n">
-        <v>14543010</v>
+        <v>13997600</v>
       </c>
       <c r="L409" s="5" t="n">
-        <v>30746</v>
+        <v>29593</v>
       </c>
       <c r="M409" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N409" s="3" t="inlineStr">
@@ -27614,18 +27614,18 @@
       </c>
       <c r="J418" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K418" s="5" t="n">
-        <v>12899670</v>
+        <v>12899600</v>
       </c>
       <c r="L418" s="5" t="n">
         <v>31009</v>
       </c>
       <c r="M418" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N418" s="3" t="inlineStr">
@@ -27808,18 +27808,18 @@
       </c>
       <c r="J421" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K421" s="5" t="n">
-        <v>14457000</v>
+        <v>13914800</v>
       </c>
       <c r="L421" s="5" t="n">
-        <v>30564</v>
+        <v>29418</v>
       </c>
       <c r="M421" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N421" s="3" t="inlineStr">
@@ -28366,18 +28366,18 @@
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K430" s="5" t="n">
-        <v>12823725</v>
+        <v>12823700</v>
       </c>
       <c r="L430" s="5" t="n">
         <v>30826</v>
       </c>
       <c r="M430" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N430" s="3" t="inlineStr">
@@ -28560,18 +28560,18 @@
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K433" s="5" t="n">
-        <v>14371905</v>
+        <v>13832900</v>
       </c>
       <c r="L433" s="5" t="n">
-        <v>30385</v>
+        <v>29245</v>
       </c>
       <c r="M433" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N433" s="3" t="inlineStr">
@@ -29118,18 +29118,18 @@
       </c>
       <c r="J442" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K442" s="5" t="n">
-        <v>12747780</v>
+        <v>12747700</v>
       </c>
       <c r="L442" s="5" t="n">
         <v>30644</v>
       </c>
       <c r="M442" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N442" s="3" t="inlineStr">
@@ -29886,18 +29886,18 @@
       </c>
       <c r="J454" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K454" s="5" t="n">
-        <v>12709350</v>
+        <v>12709300</v>
       </c>
       <c r="L454" s="5" t="n">
         <v>30551</v>
       </c>
       <c r="M454" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N454" s="3" t="inlineStr">
@@ -30654,18 +30654,18 @@
       </c>
       <c r="J466" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K466" s="5" t="n">
-        <v>12671835</v>
+        <v>12671800</v>
       </c>
       <c r="L466" s="5" t="n">
         <v>30461</v>
       </c>
       <c r="M466" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N466" s="3" t="inlineStr">
@@ -31422,18 +31422,18 @@
       </c>
       <c r="J478" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K478" s="5" t="n">
-        <v>12633405</v>
+        <v>12633400</v>
       </c>
       <c r="L478" s="5" t="n">
         <v>30369</v>
       </c>
       <c r="M478" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N478" s="3" t="inlineStr">
@@ -32190,18 +32190,18 @@
       </c>
       <c r="J490" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K490" s="5" t="n">
-        <v>12595890</v>
+        <v>12595800</v>
       </c>
       <c r="L490" s="5" t="n">
-        <v>30279</v>
+        <v>30278</v>
       </c>
       <c r="M490" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N490" s="3" t="inlineStr">
@@ -32958,18 +32958,18 @@
       </c>
       <c r="J502" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K502" s="5" t="n">
-        <v>12595890</v>
+        <v>12595800</v>
       </c>
       <c r="L502" s="5" t="n">
-        <v>30279</v>
+        <v>30278</v>
       </c>
       <c r="M502" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N502" s="3" t="inlineStr">
@@ -33152,18 +33152,18 @@
       </c>
       <c r="J505" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K505" s="5" t="n">
-        <v>14114790</v>
+        <v>14114700</v>
       </c>
       <c r="L505" s="5" t="n">
         <v>29841</v>
       </c>
       <c r="M505" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N505" s="3" t="inlineStr">
@@ -33710,18 +33710,18 @@
       </c>
       <c r="J514" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K514" s="5" t="n">
-        <v>12557460</v>
+        <v>12557400</v>
       </c>
       <c r="L514" s="5" t="n">
         <v>30186</v>
       </c>
       <c r="M514" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N514" s="3" t="inlineStr">
@@ -33904,18 +33904,18 @@
       </c>
       <c r="J517" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K517" s="5" t="n">
-        <v>14071785</v>
+        <v>13544000</v>
       </c>
       <c r="L517" s="5" t="n">
-        <v>29750</v>
+        <v>28634</v>
       </c>
       <c r="M517" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N517" s="3" t="inlineStr">
@@ -34656,18 +34656,18 @@
       </c>
       <c r="J529" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K529" s="5" t="n">
-        <v>14029695</v>
+        <v>13503400</v>
       </c>
       <c r="L529" s="5" t="n">
-        <v>29661</v>
+        <v>28548</v>
       </c>
       <c r="M529" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N529" s="3" t="inlineStr">
@@ -35214,18 +35214,18 @@
       </c>
       <c r="J538" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K538" s="5" t="n">
-        <v>12481515</v>
+        <v>12481500</v>
       </c>
       <c r="L538" s="5" t="n">
         <v>30004</v>
       </c>
       <c r="M538" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N538" s="3" t="inlineStr">
@@ -35408,18 +35408,18 @@
       </c>
       <c r="J541" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K541" s="5" t="n">
-        <v>13986690</v>
+        <v>13462100</v>
       </c>
       <c r="L541" s="5" t="n">
-        <v>29570</v>
+        <v>28461</v>
       </c>
       <c r="M541" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N541" s="3" t="inlineStr">
@@ -35966,18 +35966,18 @@
       </c>
       <c r="J550" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K550" s="5" t="n">
-        <v>12443085</v>
+        <v>12443000</v>
       </c>
       <c r="L550" s="5" t="n">
         <v>29911</v>
       </c>
       <c r="M550" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N550" s="3" t="inlineStr">
@@ -36160,18 +36160,18 @@
       </c>
       <c r="J553" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K553" s="5" t="n">
-        <v>13943685</v>
+        <v>13420700</v>
       </c>
       <c r="L553" s="5" t="n">
-        <v>29479</v>
+        <v>28374</v>
       </c>
       <c r="M553" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N553" s="3" t="inlineStr">
@@ -36718,18 +36718,18 @@
       </c>
       <c r="J562" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K562" s="5" t="n">
-        <v>12367140</v>
+        <v>12367100</v>
       </c>
       <c r="L562" s="5" t="n">
         <v>29729</v>
       </c>
       <c r="M562" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N562" s="3" t="inlineStr">
@@ -36912,18 +36912,18 @@
       </c>
       <c r="J565" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K565" s="5" t="n">
-        <v>13857675</v>
+        <v>13337900</v>
       </c>
       <c r="L565" s="5" t="n">
-        <v>29297</v>
+        <v>28199</v>
       </c>
       <c r="M565" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N565" s="3" t="inlineStr">
@@ -37470,18 +37470,18 @@
       </c>
       <c r="J574" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K574" s="5" t="n">
-        <v>12291195</v>
+        <v>12291100</v>
       </c>
       <c r="L574" s="5" t="n">
         <v>29546</v>
       </c>
       <c r="M574" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N574" s="3" t="inlineStr">
@@ -37664,18 +37664,18 @@
       </c>
       <c r="J577" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K577" s="5" t="n">
-        <v>13772580</v>
+        <v>13256000</v>
       </c>
       <c r="L577" s="5" t="n">
-        <v>29118</v>
+        <v>28025</v>
       </c>
       <c r="M577" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N577" s="3" t="inlineStr">
@@ -38222,18 +38222,18 @@
       </c>
       <c r="J586" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K586" s="5" t="n">
-        <v>12215250</v>
+        <v>12215200</v>
       </c>
       <c r="L586" s="5" t="n">
-        <v>29364</v>
+        <v>29363</v>
       </c>
       <c r="M586" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N586" s="3" t="inlineStr">
@@ -38416,18 +38416,18 @@
       </c>
       <c r="J589" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K589" s="5" t="n">
-        <v>13686570</v>
+        <v>13173200</v>
       </c>
       <c r="L589" s="5" t="n">
-        <v>28936</v>
+        <v>27850</v>
       </c>
       <c r="M589" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N589" s="3" t="inlineStr">
@@ -38974,18 +38974,18 @@
       </c>
       <c r="J598" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K598" s="5" t="n">
-        <v>12215250</v>
+        <v>12215200</v>
       </c>
       <c r="L598" s="5" t="n">
-        <v>29364</v>
+        <v>29363</v>
       </c>
       <c r="M598" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N598" s="3" t="inlineStr">
@@ -39168,18 +39168,18 @@
       </c>
       <c r="J601" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K601" s="5" t="n">
-        <v>13686570</v>
+        <v>13173200</v>
       </c>
       <c r="L601" s="5" t="n">
-        <v>28936</v>
+        <v>27850</v>
       </c>
       <c r="M601" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N601" s="3" t="inlineStr">
@@ -39726,18 +39726,18 @@
       </c>
       <c r="J610" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K610" s="5" t="n">
-        <v>12139305</v>
+        <v>12139300</v>
       </c>
       <c r="L610" s="5" t="n">
         <v>29181</v>
       </c>
       <c r="M610" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N610" s="3" t="inlineStr">
@@ -39920,18 +39920,18 @@
       </c>
       <c r="J613" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K613" s="5" t="n">
-        <v>13601475</v>
+        <v>13091300</v>
       </c>
       <c r="L613" s="5" t="n">
-        <v>28756</v>
+        <v>27677</v>
       </c>
       <c r="M613" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N613" s="3" t="inlineStr">
@@ -40478,18 +40478,18 @@
       </c>
       <c r="J622" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K622" s="5" t="n">
-        <v>12062445</v>
+        <v>12062400</v>
       </c>
       <c r="L622" s="5" t="n">
         <v>28996</v>
       </c>
       <c r="M622" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N622" s="3" t="inlineStr">
@@ -40672,18 +40672,18 @@
       </c>
       <c r="J625" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K625" s="5" t="n">
-        <v>13515465</v>
+        <v>13008500</v>
       </c>
       <c r="L625" s="5" t="n">
-        <v>28574</v>
+        <v>27502</v>
       </c>
       <c r="M625" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N625" s="3" t="inlineStr">
@@ -41230,7 +41230,7 @@
       </c>
       <c r="J634" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="K634" s="5" t="n">
@@ -41424,18 +41424,18 @@
       </c>
       <c r="J637" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>11.93%</t>
         </is>
       </c>
       <c r="K637" s="5" t="n">
-        <v>13430370</v>
+        <v>12926600</v>
       </c>
       <c r="L637" s="5" t="n">
-        <v>28394</v>
+        <v>27329</v>
       </c>
       <c r="M637" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%) + 代繳從價印花稅</t>
         </is>
       </c>
       <c r="N637" s="3" t="inlineStr">
@@ -41982,18 +41982,18 @@
       </c>
       <c r="J646" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K646" s="5" t="n">
-        <v>11872125</v>
+        <v>11872100</v>
       </c>
       <c r="L646" s="5" t="n">
         <v>28539</v>
       </c>
       <c r="M646" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N646" s="3" t="inlineStr">
@@ -42750,18 +42750,18 @@
       </c>
       <c r="J658" s="3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>8.50%</t>
         </is>
       </c>
       <c r="K658" s="5" t="n">
-        <v>11720235</v>
+        <v>11720200</v>
       </c>
       <c r="L658" s="5" t="n">
         <v>28174</v>
       </c>
       <c r="M658" s="3" t="inlineStr">
         <is>
-          <t>現金付款計劃 - 90天成交</t>
+          <t>現金付款計劃 (減8.5%)</t>
         </is>
       </c>
       <c r="N658" s="3" t="inlineStr">

</xml_diff>